<commit_message>
UPDATE #5 UI ADD
</commit_message>
<xml_diff>
--- a/FILES/sample session.xlsx
+++ b/FILES/sample session.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\visha\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\PROJECT-X\FILES\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08A34DCC-59BC-4B3A-AEC6-E79C87C99D8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{16F6E40C-7EB7-4A37-B388-87B62CBD58D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-103" yWindow="-103" windowWidth="22149" windowHeight="13200" xr2:uid="{C9880FC8-B705-4B60-AE78-C62085C5813A}"/>
   </bookViews>
@@ -27,12 +27,6 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
   <si>
-    <t>Date</t>
-  </si>
-  <si>
-    <t>SessionName</t>
-  </si>
-  <si>
     <t>Session-1</t>
   </si>
   <si>
@@ -82,6 +76,12 @@
   </si>
   <si>
     <t>General Admission-3</t>
+  </si>
+  <si>
+    <t>date</t>
+  </si>
+  <si>
+    <t>name</t>
   </si>
 </sst>
 </file>
@@ -91,7 +91,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-14009]yyyy/mm/dd;@"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -101,6 +101,14 @@
     </font>
     <font>
       <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -126,9 +134,24 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -443,174 +466,213 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BF3879BF-A08F-400F-8489-73CE5D655AB5}">
-  <dimension ref="A1:B23"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
     <col min="1" max="1" width="10.07421875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="17.921875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.3828125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.4609375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A1" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A1" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A2" s="5">
+        <v>45891</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A3" s="5">
+        <v>45891</v>
+      </c>
+      <c r="B3" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A4" s="5">
+        <v>45891</v>
+      </c>
+      <c r="B4" s="6" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A2" s="1">
-        <v>45877</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A5" s="5">
+        <v>45891</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A6" s="5">
+        <v>45891</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A7" s="5">
+        <v>45891</v>
+      </c>
+      <c r="B7" s="6" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="6"/>
+      <c r="D7" s="3"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A8" s="5">
+        <v>45892</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C8" s="6"/>
+      <c r="D8" s="3"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A9" s="5">
+        <v>45892</v>
+      </c>
+      <c r="B9" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="6"/>
+      <c r="D9" s="3"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A10" s="5">
+        <v>45892</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="6"/>
+      <c r="D10" s="3"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A11" s="5">
+        <v>45892</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11" s="6"/>
+      <c r="D11" s="3"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A12" s="5">
+        <v>45892</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C12" s="6"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A13" s="5">
+        <v>45892</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="6"/>
+      <c r="D13" s="3"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A14" s="5">
+        <v>45893</v>
+      </c>
+      <c r="B14" s="6" t="s">
         <v>16</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A3" s="1">
-        <v>45877</v>
-      </c>
-      <c r="B3" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A4" s="1">
-        <v>45877</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A5" s="1">
-        <v>45877</v>
-      </c>
-      <c r="B5" t="s">
+      <c r="C14" s="6"/>
+      <c r="D14" s="3"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A15" s="5">
+        <v>45893</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="6"/>
+      <c r="D15" s="3"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A16" s="5">
+        <v>45893</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="C16" s="6"/>
+      <c r="D16" s="3"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A17" s="5">
+        <v>45893</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17" s="6"/>
+      <c r="D17" s="3"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+      <c r="A18" s="5">
+        <v>45893</v>
+      </c>
+      <c r="B18" s="6" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A6" s="1">
-        <v>45877</v>
-      </c>
-      <c r="B6" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A7" s="1">
-        <v>45877</v>
-      </c>
-      <c r="B7" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A8" s="1">
-        <v>45878</v>
-      </c>
-      <c r="B8" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A9" s="1">
-        <v>45878</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A10" s="1">
-        <v>45878</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A11" s="1">
-        <v>45878</v>
-      </c>
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A12" s="1">
-        <v>45878</v>
-      </c>
-      <c r="B12" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A13" s="1">
-        <v>45878</v>
-      </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A14" s="1">
-        <v>45879</v>
-      </c>
-      <c r="B14" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A15" s="1">
-        <v>45879</v>
-      </c>
-      <c r="B15" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A16" s="1">
-        <v>45879</v>
-      </c>
-      <c r="B16" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A17" s="1">
-        <v>45879</v>
-      </c>
-      <c r="B17" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.4">
-      <c r="A18" s="1">
-        <v>45879</v>
-      </c>
-      <c r="B18" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.4">
+      <c r="C18" s="6"/>
+      <c r="D18" s="3"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A19" s="1"/>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A20" s="1"/>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
       <c r="A23" s="1"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>